<commit_message>
Completed Analysis Module and added Aadhaar No. field in students upload
</commit_message>
<xml_diff>
--- a/public/uploads/sample/bulk_students_sample_file.xlsx
+++ b/public/uploads/sample/bulk_students_sample_file.xlsx
@@ -1,28 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20416"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr showInkAnnotation="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\wamp64\www\projects\uatassmt\public\uploads\sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FC9DC18-E6CE-4F0A-BCC8-F12F7D2A1ADE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67D8E34B-26F7-41AF-92E1-E24B1A927495}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="32760" yWindow="32760" windowWidth="20385" windowHeight="8370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="52">
   <si>
     <t>Name of Training Agency</t>
   </si>
@@ -175,6 +173,9 @@
   </si>
   <si>
     <t>dw</t>
+  </si>
+  <si>
+    <t>Aadhaar No</t>
   </si>
 </sst>
 </file>
@@ -567,7 +568,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" bestFit="1" customWidth="1"/>
@@ -584,7 +585,7 @@
     <col min="12" max="12" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="11" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="23" customWidth="1"/>
     <col min="16" max="16" width="21.5703125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="49.5703125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="9.85546875" bestFit="1" customWidth="1"/>
@@ -614,7 +615,7 @@
     <col min="42" max="42" width="7.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="3" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" s="3" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>42</v>
       </c>
@@ -657,8 +658,11 @@
       <c r="N1" s="2" t="s">
         <v>6</v>
       </c>
+      <c r="O1" s="2" t="s">
+        <v>51</v>
+      </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>48</v>
       </c>
@@ -695,8 +699,11 @@
       <c r="N2">
         <v>9100101100</v>
       </c>
+      <c r="O2">
+        <v>123456789112</v>
+      </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>48</v>
       </c>
@@ -733,8 +740,11 @@
       <c r="N3">
         <v>9100101101</v>
       </c>
+      <c r="O3">
+        <v>123456789112</v>
+      </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>49</v>
       </c>
@@ -771,8 +781,11 @@
       <c r="N4">
         <v>9100101102</v>
       </c>
+      <c r="O4">
+        <v>123456789112</v>
+      </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>49</v>
       </c>
@@ -809,8 +822,11 @@
       <c r="N5">
         <v>9100101103</v>
       </c>
+      <c r="O5">
+        <v>123456789112</v>
+      </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>48</v>
       </c>
@@ -847,8 +863,11 @@
       <c r="N6">
         <v>9100101104</v>
       </c>
+      <c r="O6">
+        <v>123456789112</v>
+      </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>48</v>
       </c>
@@ -885,8 +904,11 @@
       <c r="N7">
         <v>9100101105</v>
       </c>
+      <c r="O7">
+        <v>123456789112</v>
+      </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>49</v>
       </c>
@@ -923,8 +945,11 @@
       <c r="N8">
         <v>9100101106</v>
       </c>
+      <c r="O8">
+        <v>123456789112</v>
+      </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>48</v>
       </c>
@@ -961,8 +986,11 @@
       <c r="N9">
         <v>9100101107</v>
       </c>
+      <c r="O9">
+        <v>123456789112</v>
+      </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>48</v>
       </c>
@@ -1000,7 +1028,7 @@
         <v>9100101108</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>48</v>
       </c>
@@ -1036,28 +1064,13 @@
       </c>
       <c r="N11">
         <v>9100101109</v>
+      </c>
+      <c r="O11">
+        <v>123456789112</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>